<commit_message>
adding obs at TERCEIROS
</commit_message>
<xml_diff>
--- a/modelo_mapinfo_nf3.xlsx
+++ b/modelo_mapinfo_nf3.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\NFV 3.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\F257064\Documents\Codes\NFV 3.0\NFV 3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{033A7A20-A081-4D5B-91A2-573B7208F90A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F3C0E37-835E-4D42-950B-3F121D97F1C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="arquivo_mapinfo_orc_02_04_2025_" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" iterateDelta="1E-4"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="109">
   <si>
     <t>SEV</t>
   </si>
@@ -41,6 +41,312 @@
   </si>
   <si>
     <t>VTAL3K</t>
+  </si>
+  <si>
+    <t>0.037429500</t>
+  </si>
+  <si>
+    <t>-12.1415715</t>
+  </si>
+  <si>
+    <t>-44.9899657</t>
+  </si>
+  <si>
+    <t>-16.6895471</t>
+  </si>
+  <si>
+    <t>-49.2309077</t>
+  </si>
+  <si>
+    <t>-19.5397700</t>
+  </si>
+  <si>
+    <t>-40.6385797</t>
+  </si>
+  <si>
+    <t>-6.07453990</t>
+  </si>
+  <si>
+    <t>-49.8717520</t>
+  </si>
+  <si>
+    <t>-9.77178400</t>
+  </si>
+  <si>
+    <t>-36.6508100</t>
+  </si>
+  <si>
+    <t>-3.84179789</t>
+  </si>
+  <si>
+    <t>-38.4865220</t>
+  </si>
+  <si>
+    <t>-51.0705955</t>
+  </si>
+  <si>
+    <t>-22.7990601</t>
+  </si>
+  <si>
+    <t>-43.4193744</t>
+  </si>
+  <si>
+    <t>-5.75454080</t>
+  </si>
+  <si>
+    <t>-35.2804842</t>
+  </si>
+  <si>
+    <t>-19.5722700</t>
+  </si>
+  <si>
+    <t>-46.9405100</t>
+  </si>
+  <si>
+    <t>-20.3448664</t>
+  </si>
+  <si>
+    <t>-40.3299510</t>
+  </si>
+  <si>
+    <t>-2.55226566</t>
+  </si>
+  <si>
+    <t>-44.2598188</t>
+  </si>
+  <si>
+    <t>-17.8780598</t>
+  </si>
+  <si>
+    <t>-51.7228171</t>
+  </si>
+  <si>
+    <t>-20.3347238</t>
+  </si>
+  <si>
+    <t>-40.3342266</t>
+  </si>
+  <si>
+    <t>-22.9067432</t>
+  </si>
+  <si>
+    <t>-43.2419590</t>
+  </si>
+  <si>
+    <t>-29.1369600</t>
+  </si>
+  <si>
+    <t>-56.5366700</t>
+  </si>
+  <si>
+    <t>-16.3208055</t>
+  </si>
+  <si>
+    <t>-48.9636368</t>
+  </si>
+  <si>
+    <t>-22.8652964</t>
+  </si>
+  <si>
+    <t>-43.2732388</t>
+  </si>
+  <si>
+    <t>-29.4893809</t>
+  </si>
+  <si>
+    <t>-51.9686631</t>
+  </si>
+  <si>
+    <t>-8.04142340</t>
+  </si>
+  <si>
+    <t>-34.8804852</t>
+  </si>
+  <si>
+    <t>-4.86382840</t>
+  </si>
+  <si>
+    <t>-43.3580040</t>
+  </si>
+  <si>
+    <t>-22.8470103</t>
+  </si>
+  <si>
+    <t>-43.3743925</t>
+  </si>
+  <si>
+    <t>-16.6061651</t>
+  </si>
+  <si>
+    <t>-49.3354645</t>
+  </si>
+  <si>
+    <t>-15.4917310</t>
+  </si>
+  <si>
+    <t>-47.1075546</t>
+  </si>
+  <si>
+    <t>-29.4637707</t>
+  </si>
+  <si>
+    <t>-51.7766080</t>
+  </si>
+  <si>
+    <t>-29.6012516</t>
+  </si>
+  <si>
+    <t>-52.2124400</t>
+  </si>
+  <si>
+    <t>-16.3667206</t>
+  </si>
+  <si>
+    <t>-39.5750880</t>
+  </si>
+  <si>
+    <t>-11.8331500</t>
+  </si>
+  <si>
+    <t>-55.5152500</t>
+  </si>
+  <si>
+    <t>-22.2924000</t>
+  </si>
+  <si>
+    <t>-42.5263500</t>
+  </si>
+  <si>
+    <t>-22.5428300</t>
+  </si>
+  <si>
+    <t>-43.5749416</t>
+  </si>
+  <si>
+    <t>-13.8667427</t>
+  </si>
+  <si>
+    <t>-40.0750580</t>
+  </si>
+  <si>
+    <t>-22.9748734</t>
+  </si>
+  <si>
+    <t>-46.9830902</t>
+  </si>
+  <si>
+    <t>-22.7766004</t>
+  </si>
+  <si>
+    <t>-43.4403304</t>
+  </si>
+  <si>
+    <t>-22.6801659</t>
+  </si>
+  <si>
+    <t>-47.6589263</t>
+  </si>
+  <si>
+    <t>-22.4206316</t>
+  </si>
+  <si>
+    <t>-47.5631848</t>
+  </si>
+  <si>
+    <t>-23.3027281</t>
+  </si>
+  <si>
+    <t>-46.2171135</t>
+  </si>
+  <si>
+    <t>-22.3804832</t>
+  </si>
+  <si>
+    <t>-47.5716623</t>
+  </si>
+  <si>
+    <t>-26.2729583</t>
+  </si>
+  <si>
+    <t>-49.3958867</t>
+  </si>
+  <si>
+    <t>-23.4024000</t>
+  </si>
+  <si>
+    <t>-46.4477700</t>
+  </si>
+  <si>
+    <t>-25.5957098</t>
+  </si>
+  <si>
+    <t>-49.3895229</t>
+  </si>
+  <si>
+    <t>-27.0102083</t>
+  </si>
+  <si>
+    <t>-51.1623245</t>
+  </si>
+  <si>
+    <t>-25.5341660</t>
+  </si>
+  <si>
+    <t>-48.5113297</t>
+  </si>
+  <si>
+    <t>-16.6786981</t>
+  </si>
+  <si>
+    <t>-49.3889855</t>
+  </si>
+  <si>
+    <t>-29.1662152</t>
+  </si>
+  <si>
+    <t>-51.5020630</t>
+  </si>
+  <si>
+    <t>-3.81367170</t>
+  </si>
+  <si>
+    <t>-38.4314117</t>
+  </si>
+  <si>
+    <t>-27.5479702</t>
+  </si>
+  <si>
+    <t>-48.4947071</t>
+  </si>
+  <si>
+    <t>-16.7326526</t>
+  </si>
+  <si>
+    <t>-49.2283898</t>
+  </si>
+  <si>
+    <t>-8.04386333</t>
+  </si>
+  <si>
+    <t>-34.8772416</t>
+  </si>
+  <si>
+    <t>-3.89210940</t>
+  </si>
+  <si>
+    <t>-38.4361896</t>
+  </si>
+  <si>
+    <t>-16.6732033</t>
+  </si>
+  <si>
+    <t>-49.2408697</t>
+  </si>
+  <si>
+    <t>-16.6458087</t>
+  </si>
+  <si>
+    <t>-49.2780576</t>
   </si>
 </sst>
 </file>
@@ -524,9 +830,12 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -850,7 +1159,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.77734375" style="1" bestFit="1" customWidth="1"/>
@@ -882,6 +1191,567 @@
         <v>6</v>
       </c>
     </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>8845407</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>8845408</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>8845411</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>8845416</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>8845447</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>8845451</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>8845470</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>8845476</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="1">
+        <v>8845489</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="1">
+        <v>8845491</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="1">
+        <v>8845510</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="1">
+        <v>8845513</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="1">
+        <v>8845555</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="1">
+        <v>8845577</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="1">
+        <v>8845579</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1">
+        <v>8845581</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="1">
+        <v>8845587</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>8845589</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>8845599</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>8845600</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>8845693</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>8845695</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>8845702</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>8845704</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>8845706</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>8845707</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>8845759</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>8845760</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="1">
+        <v>8845762</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="1">
+        <v>8845766</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="1">
+        <v>8845768</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>8845771</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>8845774</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>8845775</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>8845786</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>8845790</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>8845792</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>8845799</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>8845800</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>8845810</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>8845811</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>8845812</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="1">
+        <v>8845816</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="1">
+        <v>8845817</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="1">
+        <v>8845821</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="1">
+        <v>8845824</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="1">
+        <v>8845830</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="1">
+        <v>8845831</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="1">
+        <v>8845834</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="1">
+        <v>8845835</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="1">
+        <v>8845839</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>